<commit_message>
Use only disclosed financing classifications
</commit_message>
<xml_diff>
--- a/HTG_Financing_Review.xlsx
+++ b/HTG_Financing_Review.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf1270510086c4148"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding" sheetId="2" r:id="R3f6565be4c2f4a91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R4dec65a48cb644b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc1a066955154463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding" sheetId="2" r:id="Rd8a0004f99204696"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R96b74dfa40b64e6d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -531,7 +531,7 @@
         <x:v>Rainbow Village</x:v>
       </x:c>
       <x:c r="B6" s="1" t="str">
-        <x:v>subordinate_debt</x:v>
+        <x:v>program_financing</x:v>
       </x:c>
       <x:c r="C6" s="1" t="str">
         <x:v>SAIL financing</x:v>
@@ -540,7 +540,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E6" s="1" t="str">
-        <x:v>Rainbow Village|subordinate_debt</x:v>
+        <x:v>Rainbow Village|program_financing</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -616,7 +616,7 @@
         <x:v>Rainbow Village</x:v>
       </x:c>
       <x:c r="B11" s="1" t="str">
-        <x:v>subordinate_debt</x:v>
+        <x:v>seller_note</x:v>
       </x:c>
       <x:c r="C11" s="1" t="str">
         <x:v>PHCD seller note</x:v>
@@ -625,7 +625,7 @@
         <x:v>3.1</x:v>
       </x:c>
       <x:c r="E11" s="1" t="str">
-        <x:v>Rainbow Village|subordinate_debt</x:v>
+        <x:v>Rainbow Village|seller_note</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -633,7 +633,7 @@
         <x:v>Rainbow Village</x:v>
       </x:c>
       <x:c r="B12" s="1" t="str">
-        <x:v>subordinate_debt</x:v>
+        <x:v>public_loan</x:v>
       </x:c>
       <x:c r="C12" s="1" t="str">
         <x:v>PHCD HOME loan</x:v>
@@ -642,7 +642,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E12" s="1" t="str">
-        <x:v>Rainbow Village|subordinate_debt</x:v>
+        <x:v>Rainbow Village|public_loan</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -650,7 +650,7 @@
         <x:v>Rainbow Village</x:v>
       </x:c>
       <x:c r="B13" s="1" t="str">
-        <x:v>subordinate_debt</x:v>
+        <x:v>public_loan</x:v>
       </x:c>
       <x:c r="C13" s="1" t="str">
         <x:v>SEOPW CRA loan</x:v>
@@ -659,7 +659,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E13" s="1" t="str">
-        <x:v>Rainbow Village|subordinate_debt</x:v>
+        <x:v>Rainbow Village|public_loan</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -735,7 +735,7 @@
         <x:v>Artisan Pointe Phase I</x:v>
       </x:c>
       <x:c r="B18" s="1" t="str">
-        <x:v>subordinate_debt</x:v>
+        <x:v>public_loan</x:v>
       </x:c>
       <x:c r="C18" s="1" t="str">
         <x:v>Naranja Lakes CRA loan</x:v>
@@ -744,7 +744,7 @@
         <x:v>3.5</x:v>
       </x:c>
       <x:c r="E18" s="1" t="str">
-        <x:v>Artisan Pointe Phase I|subordinate_debt</x:v>
+        <x:v>Artisan Pointe Phase I|public_loan</x:v>
       </x:c>
     </x:row>
     <x:row r="19">

</xml_diff>